<commit_message>
Rewrite Sugar News 2026-07-31 report
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-31.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-31.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -513,12 +513,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>ChiniMandi消息涉及巴西食糖价格或市场流通变化。价格变化会影响贸易商采购、终端补库和政策调控预期，对短期糖价走势具有参考意义。来源：ChiniMandi（https://news.google.com/rss/articles/CBMitAFBVV95cUxPMWhNS09VYVF1cHljWmloYUMzS3BZWFZSdUNFRzRyM2xQVjRmdTRUZzdHNHozeHZhb1Y5QUNvWHNDQThLVk1ybmZqdDZibENUS01zVWJKTE1MSGpBemxkMDJ5bWN3b0FCQXZQSlpGWXJrUFNaSjUza2MzRFYyZzhqN1JNQjhJVGJjRm9Xb1J6ZkJka1ZlaEFSbDlzZU9GellCbE5hTlF5QWplYURGMnAwV0tVUjA?oc=5）</t>
+          <t>Czarnikow Group分析负责人Stephen Geldart表示，2026年全球原糖仍有大量过剩，过剩糖正在巴西中南部生产，巴西预计占全球原糖供应的72%。他同时指出，全球食糖消费量约为1.78亿吨，较2014年前2%年增速趋势下的2.08亿吨少3000万吨，需求放缓叠加巴西玉米乙醇占乙醇产量超过25%，会削弱甘蔗转乙醇对糖价的缓冲，因此利空原糖。来源：ChiniMandi（https://www.chinimandi.com/the-biggest-threat-to-sugar-prices-isnt-supply-its-slowing-consumption-stephen-geldart/）</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>利空：巴西供应占比抬高且全球消费缺口扩大，会增加原糖库存和出口压力，从而压制国际原糖价格。</t>
         </is>
       </c>
     </row>
@@ -530,12 +530,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>kathmandupost.com消息涉及印度食糖贸易、关税或配额安排。进出口政策和贸易流向变化会改变国内外可用糖源，对区域供应和国际糖价形成影响。来源：kathmandupost.com（https://news.google.com/rss/articles/CBMiswFBVV95cUxOWkQxM09ROXAxUDViS3BRTXNNbHUyMTBoX3NvNWRoT3FTeFZSX3hhMDdVajNpeTNjT3lPZ21mUHdVdlNXdXZMX3pKQlJ5QS1PQi02T1QxUy1NLUc4VlRSdzNFMktjcnRMU0xsR3Vaal8xZ0xMYzgzcUkxTGFUSTZrYnZNa0NBd0E5TzBtU2szUjI5VUpfVFM3T0ZhcG15VHJETnY5NTNwSFVablhPSDczNWZqNA?oc=5）</t>
+          <t>尼泊尔武装警察部队称，印度5月13日至9月30日禁止食糖出口后，尼泊尔南部边境6月中至7月中查获走私糖10吨、价值780255尼泊尔卢比，前一月为4吨、284870尼泊尔卢比。尼泊尔零售糖价由约95卢比/公斤涨至约110卢比/公斤，印度出口禁令减少正规进口可得糖源并推升节前补库压力，因此利多南亚区域现货糖价。来源：The Kathmandu Post（https://kathmandupost.com/money/2026/07/31/india-s-sugar-export-ban-fuels-smuggling-ahead-of-peak-festival-season）</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>偏多糖价：贸易限制或供应扰动可能减少国际市场可用糖源。</t>
+          <t>偏多糖价：印度限制出口使尼泊尔正规进口供应减少，节前需求增加会放大库存紧张，从而支撑区域食糖价格。</t>
         </is>
       </c>
     </row>
@@ -547,148 +547,63 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>timesofindia.indiatimes.com消息涉及印度糖厂、甘蔗或甜菜生产环节变化。相关变化可能影响糖料供应、压榨节奏或加工能力，后续需跟踪对食糖产量和现货供应的实际影响。来源：timesofindia.indiatimes.com（https://news.google.com/rss/articles/CBMi0gFBVV95cUxQVmd1UnFqN3NxQWpnSUxFb0VCMUdCeUxFMlFIVEhoNHZQX3lNMFBtOVkxWkRDM2FZVFktb0wwQjlUM3RpNWdfQ2p1LTI4RXEyQ092Q0sxdVZqT3JyaklZNnZxTEozajZNZ3U1YVloRFlzU3BoWnVNNTlvWlk4aEFIRjk1Q0tsU20zLXdaSGdBeDdadDBCTFIycVJlcVlEMlZtMTdyY2ZXbzROTlg4YVk0V3dyOG81WXhzTVl6SkpaUUNmV3E1QU9XZEU3OHl4cEdqdmfSAdIBQVVfeXFMUFZndVJxajdzcUFqZ0lMRW9FQjFHQnlMRTJRSFRIaDR2UF95TTBQbTlZMVpEQzNhWVRZLW9MMEI5VDN0aTVnX0NqdS0yOEVxMkNPdkNLMXVWak9ycmpJWTZ2cUxKM2o2TWd1NWFZaERZc1NwaFp1TTU5b1pZOGhBSEY5NUNLbFNtMy13WkhnQXg3WnQwQkxSMnFSZXFZRDJWbTE3cmNmV280Tk5YOGFZNFd3cjhvNVl4c01ZekpKWlFDZldxNUFPV2RFNzh5eHBHanZn?oc=5）</t>
+          <t>印度全国合作糖厂联合会（NFCSF）和印度糖厂协会（ISMA）宣布在哥印拜陀ICAR-SBI建设甘蔗卓越中心，行业计划出资4.5亿卢比，中央政府预计再出资约4.5亿卢比，总投资9亿卢比。该中心将研发高单产、高出糖率以及抗旱、抗涝、耐盐和耐热甘蔗品种，以缓解印度糖厂压榨季由150—160天缩短至约100天的原料不足，中长期提高糖料供应和产糖潜力，利空远期糖价。来源：The Times of India（https://timesofindia.indiatimes.com/city/coimbatore/rs-90crore-sugarcane-rd-hub-to-be-set-up-in-coimbatore/amp_articleshow/132769124.cms）</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>偏空糖价：研发投入若提高甘蔗单产和出糖率，会增加印度糖料供应和制糖潜力，从而压制远期食糖价格；短期对当季供应影响有限。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="180" customHeight="1" s="2">
+    <row r="5" ht="110.9" customHeight="1" s="2">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>AgroSpectrum India消息涉及印度乙醇、糖蜜或糖料分流安排。若甘蔗、糖蜜或糖浆更多流向制醇，可能减少制糖供应；反之则可能增加食糖产出。来源：AgroSpectrum India（https://news.google.com/rss/articles/CBMiqwFBVV95cUxNcE5kZmJuLS12VlhHUVhNVGRYVG1KVEhtbVBaaDlMaTdqbF8tMGJXaU1TX3hFWUd1YmN0a3RNTTJRbk5rdk5icHpackNsVzJNaFI3aExHampBZlE4d2F3Q05tMWNmWnhMWGhFU1FvYTluT0lCVm8wc19lNG9LX1pJVFRjeWg1Vlc2c3d5ellNWkFmTDBkRk5pQ29VQTJhV2V5MjQ4QWozbm5WbTg?oc=5）</t>
+          <t>泰国气象局预报（2026-07-31），乌隆他尼、黎府、甘烹碧、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，雷阵雨和局地大雨有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>偏多糖价：乙醇需求或政策推进可能增加糖料制醇吸引力，减少部分制糖供应。</t>
+          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="180" customHeight="1" s="2">
+    <row r="6" ht="118.05" customHeight="1" s="2">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>中国</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>The Indian Awaaz消息涉及印度糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：The Indian Awaaz（https://news.google.com/rss/articles/CBMimAFBVV95cUxOMVMtdDVXMlMtYjdaMnVGVE1vM2syUHFRdmFiZnd1U1YzalVEUUhpdkVwWXduWXI2Z2hETERFc1NoWVVhYzVtTkZkaGRBci1DdEl6X3dTc3AzcmNCbnc4bVRNMkg2S1F5NmRFaWg2VF90eENjODJudjZSWWNQMjVqM29aMmpKdk5zdl9ua1djUk1VRExHbkZqVA?oc=5）</t>
+          <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="180" customHeight="1" s="2">
+    <row r="7" ht="135.65" customHeight="1" s="2">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>肯尼亚</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Nikkei Asia消息涉及印度糖厂、甘蔗或甜菜生产环节变化。相关变化可能影响糖料供应、压榨节奏或加工能力，后续需跟踪对食糖产量和现货供应的实际影响。来源：Nikkei Asia（https://news.google.com/rss/articles/CBMiqgFBVV95cUxPZjRkM1JXNV9zRGFZckktLWgwZGtPeklsWktHYWVKZHl6WGJVa1RSY2lKbDdDeVBuU0lfVHpEM19iTGI3cEw1Z0N0ejhNRFZnU0lBeWFxNlE1SE9kOEN6VTlDQXBaLXJHSjVRdU1WZWE0b0l5ckdfd3hGcGk2ODgtWFlkQlA1cF8xZVlSdXNGMDNuVU1SYWd3RFIwMXZQZlRBWHd2QTNKSUtHQQ?oc=5）</t>
+          <t>肯尼亚农业首席秘书Kipronoh Ronoh禁止本地糖厂进口食糖，称肯尼亚月度产糖已由约4万吨增加至超过8万吨，足以满足国内需求。该禁令要求糖厂优先压榨本地甘蔗并消化库存，减轻进口糖对本地糖厂和蔗农的竞争；由于肯尼亚进口规模有限，对国际糖价影响有限。来源：The Kenyan Wallstreet（https://kenyanwallstreet.com/local-cane-ban-imports）</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="180" customHeight="1" s="2">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>泰国</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Houston Press消息涉及泰国糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：Houston Press（https://news.google.com/rss/articles/CBMipAFBVV95cUxNRGJjUExha2xwNnhxNGhuMERoQ0huVU1qTjV1OTBaQVRsRXNORmxqYUw1UmdydlVVdWlaRjV3SjJDSnpTcEozb1EwN2IzN1U5NHFrZ1Zpb3RFYkV0RHpTN1dBelR6TVNrSE5JVnQzMTZsNVBrMjdTd1dVQ0RxOU9CUGtfM1JnbEp0TmlKLWlBUHk2TWNvWmJkcjlKSGtJZ3ZTajU1bA?oc=5）</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="180" customHeight="1" s="2">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>泰国</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>kashmirage.net消息涉及泰国糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：kashmirage.net（https://news.google.com/rss/articles/CBMihAFBVV95cUxQVlFBSGtoVDFkNWtVV0wzZ09DUjg4R0tVMzM4WGtXWjc4SmpuQi1OYm5WN1pjQVhGUnZ5aFNhb3F1SjdZc2JaczJWdm5tSHVmMW1oN0JpR1VDMk9SbFNFRUJUci1mVktLYnNZVnhRYWpYb0V1Y1RfNHNyWVdKa29oV0VNVUc?oc=5）</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="114.2" customHeight="1" s="2">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>泰国</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>泰国气象局预报（2026-07-31），乌隆他尼、黎府、甘烹碧、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="118.05" customHeight="1" s="2">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>中国</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="175.25" customHeight="1" s="2">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>肯尼亚</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>The Kenyan Wallstreet消息涉及肯尼亚糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：The Kenyan Wallstreet（https://news.google.com/rss/articles/CBMiYEFVX3lxTFBLMkFYREw0RGt6a0tubGdrVGNONnFOTldMX0tCMndVMmdPdmV1Y3h4WE9BekEydDQ1em5UUXhPUTlnLW9nT3JnMzZhX3ZSOVpzWEJMM3ZsOC1NcHM3S2ZHQg?oc=5）</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>影响有限：肯尼亚产糖增加会减少进口需求并补充本地供应，但其贸易体量不足以明显改变全球食糖供需，因此对国际糖价影响有限。</t>
         </is>
       </c>
     </row>

</xml_diff>